<commit_message>
Add MEP savings to APC Filigree budget
Additional savings from MEP embedding:
- Electrical: 10% savings (.31/SF) - conduits pre-laid on precast before topping
- Plumbing: 10% savings (.88/SF) - pipes sandwiched between precast and topping
- Total additional savings: ~

Updated RFQ:
- Added MEP embedding to benefits list
- Added MEP conduit/pipe pre-lay as scope item (.75/SF)
- Notes explain how conduits/pipes are laid on precast then encased in topping slab

This sandwich system reduces electrician and plumber labor significantly
</commit_message>
<xml_diff>
--- a/NEVO_Tower/outputs/NEVO_APC_Budget.xlsx
+++ b/NEVO_Tower/outputs/NEVO_APC_Budget.xlsx
@@ -36420,7 +36420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36561,167 +36561,117 @@
     <row r="20">
       <c r="A20" s="98" t="inlineStr">
         <is>
-          <t>✓ Improved quality control (factory fabrication)</t>
+          <t>✓ MEP conduits/pipes embedded between precast and topping slab</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="98" t="inlineStr">
         <is>
-          <t>✓ Reduced concrete waste and material costs</t>
+          <t>✓ 10% savings on electrical and plumbing (pre-laid before pour)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="98" t="inlineStr">
         <is>
-          <t>✓ Integrated structural steel support system</t>
+          <t>✓ Improved quality control (factory fabrication)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="98" t="inlineStr">
         <is>
-          <t>✓ Fire-rated and code-compliant</t>
+          <t>✓ Reduced concrete waste and material costs</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="98" t="inlineStr">
         <is>
+          <t>✓ Integrated structural steel support system</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="98" t="inlineStr">
+        <is>
+          <t>✓ Fire-rated and code-compliant</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="98" t="inlineStr">
+        <is>
           <t>✓ Suitable for high-rise construction</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="18" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="18" t="inlineStr">
         <is>
           <t>SCOPE OF WORK - APC FILIGREE SYSTEM</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="18" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="18" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B27" s="18" t="inlineStr">
+      <c r="B29" s="18" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C27" s="18" t="inlineStr">
+      <c r="C29" s="18" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="D27" s="18" t="inlineStr">
+      <c r="D29" s="18" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="E27" s="18" t="inlineStr">
+      <c r="E29" s="18" t="inlineStr">
         <is>
           <t>Unit Price</t>
         </is>
       </c>
-      <c r="F27" s="18" t="inlineStr">
+      <c r="F29" s="18" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="G27" s="18" t="inlineStr">
+      <c r="G29" s="18" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>APC Filigree Deck Panels</t>
-        </is>
-      </c>
-      <c r="C28" s="99" t="n">
-        <v>108675</v>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>SF</t>
-        </is>
-      </c>
-      <c r="E28" s="9" t="n">
-        <v>28.5</v>
-      </c>
-      <c r="F28" s="3">
-        <f>C28*E28</f>
-        <v/>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>Factory fabricated</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Structural Steel Integration</t>
-        </is>
-      </c>
-      <c r="C29" s="99" t="n">
-        <v>108675</v>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>SF</t>
-        </is>
-      </c>
-      <c r="E29" s="9" t="n">
-        <v>3.08</v>
-      </c>
-      <c r="F29" s="3">
-        <f>C29*E29</f>
-        <v/>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>Embedded supports</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Topping Concrete</t>
+          <t>APC Filigree Deck Panels</t>
         </is>
       </c>
       <c r="C30" s="99" t="n">
-        <v>27168.75</v>
+        <v>108675</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>CY</t>
+          <t>SF</t>
         </is>
       </c>
       <c r="E30" s="9" t="n">
-        <v>200</v>
+        <v>28.5</v>
       </c>
       <c r="F30" s="3">
         <f>C30*E30</f>
@@ -36729,19 +36679,19 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>3" topping slab</t>
+          <t>Factory fabricated</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Panel Installation Labor</t>
+          <t>Structural Steel Integration</t>
         </is>
       </c>
       <c r="C31" s="99" t="n">
@@ -36753,7 +36703,7 @@
         </is>
       </c>
       <c r="E31" s="9" t="n">
-        <v>2.5</v>
+        <v>3.08</v>
       </c>
       <c r="F31" s="3">
         <f>C31*E31</f>
@@ -36761,23 +36711,23 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Crane &amp; crew</t>
+          <t>Embedded supports</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Shoring (minimal)</t>
+          <t>MEP Conduit/Pipe Pre-Lay</t>
         </is>
       </c>
       <c r="C32" s="99" t="n">
-        <v>21735</v>
+        <v>108675</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -36785,7 +36735,7 @@
         </is>
       </c>
       <c r="E32" s="9" t="n">
-        <v>1.5</v>
+        <v>0.75</v>
       </c>
       <c r="F32" s="3">
         <f>C32*E32</f>
@@ -36793,31 +36743,31 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Temporary only</t>
+          <t>Before topping pour</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Connections &amp; Anchors</t>
+          <t>Topping Concrete</t>
         </is>
       </c>
       <c r="C33" s="99" t="n">
-        <v>350</v>
+        <v>27168.75</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>EA</t>
+          <t>CY</t>
         </is>
       </c>
       <c r="E33" s="9" t="n">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="F33" s="3">
         <f>C33*E33</f>
@@ -36825,31 +36775,31 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Per floor connections</t>
+          <t>3" topping slab</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Engineering &amp; Shop Drawings</t>
+          <t>Panel Installation Labor</t>
         </is>
       </c>
       <c r="C34" s="99" t="n">
-        <v>1</v>
+        <v>108675</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>LS</t>
+          <t>SF</t>
         </is>
       </c>
       <c r="E34" s="9" t="n">
-        <v>45000</v>
+        <v>2.5</v>
       </c>
       <c r="F34" s="3">
         <f>C34*E34</f>
@@ -36857,31 +36807,31 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Structural PE</t>
+          <t>Crane &amp; crew</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Transportation &amp; Delivery</t>
+          <t>Shoring (minimal)</t>
         </is>
       </c>
       <c r="C35" s="99" t="n">
-        <v>108.675</v>
+        <v>21735</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Loads</t>
+          <t>SF</t>
         </is>
       </c>
       <c r="E35" s="9" t="n">
-        <v>2500</v>
+        <v>1.5</v>
       </c>
       <c r="F35" s="3">
         <f>C35*E35</f>
@@ -36889,31 +36839,31 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Per truck</t>
+          <t>Temporary only</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Crane Time</t>
+          <t>Connections &amp; Anchors</t>
         </is>
       </c>
       <c r="C36" s="99" t="n">
-        <v>90</v>
+        <v>350</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Days</t>
+          <t>EA</t>
         </is>
       </c>
       <c r="E36" s="9" t="n">
-        <v>1200</v>
+        <v>250</v>
       </c>
       <c r="F36" s="3">
         <f>C36*E36</f>
@@ -36921,19 +36871,19 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Tower crane rental</t>
+          <t>Per floor connections</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Quality Control &amp; Testing</t>
+          <t>Engineering &amp; Shop Drawings</t>
         </is>
       </c>
       <c r="C37" s="99" t="n">
@@ -36945,7 +36895,7 @@
         </is>
       </c>
       <c r="E37" s="9" t="n">
-        <v>25000</v>
+        <v>45000</v>
       </c>
       <c r="F37" s="3">
         <f>C37*E37</f>
@@ -36953,260 +36903,358 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
+          <t>Structural PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Transportation &amp; Delivery</t>
+        </is>
+      </c>
+      <c r="C38" s="99" t="n">
+        <v>108.675</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Loads</t>
+        </is>
+      </c>
+      <c r="E38" s="9" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F38" s="3">
+        <f>C38*E38</f>
+        <v/>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Per truck</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Crane Time</t>
+        </is>
+      </c>
+      <c r="C39" s="99" t="n">
+        <v>90</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Days</t>
+        </is>
+      </c>
+      <c r="E39" s="9" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F39" s="3">
+        <f>C39*E39</f>
+        <v/>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Tower crane rental</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Quality Control &amp; Testing</t>
+        </is>
+      </c>
+      <c r="C40" s="99" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>LS</t>
+        </is>
+      </c>
+      <c r="E40" s="9" t="n">
+        <v>25000</v>
+      </c>
+      <c r="F40" s="3">
+        <f>C40*E40</f>
+        <v/>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
           <t>Third party</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="B38" s="17" t="inlineStr">
+    <row r="41">
+      <c r="B41" s="17" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="F38" s="24">
-        <f>SUM(F28:F37)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="18" t="inlineStr">
+      <c r="F41" s="24">
+        <f>SUM(F30:F40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="18" t="inlineStr">
         <is>
           <t>CONSTRUCTION SCHEDULE</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="17" t="inlineStr">
-        <is>
-          <t>Phase 1</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Shop Drawings &amp; Fabrication</t>
-        </is>
-      </c>
-      <c r="E42" s="17" t="inlineStr">
-        <is>
-          <t>2 months</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>Before on-site work</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="17" t="inlineStr">
-        <is>
-          <t>Phase 2</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Foundation &amp; Columns</t>
-        </is>
-      </c>
-      <c r="E43" s="17" t="inlineStr">
-        <is>
-          <t>3 months</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>Concurrent with fabrication</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="17" t="inlineStr">
-        <is>
-          <t>Phase 3</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Deck Installation (7 floors)</t>
-        </is>
-      </c>
-      <c r="E44" s="17" t="inlineStr">
-        <is>
-          <t>9 months</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>1.3 months per floor</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="17" t="inlineStr">
         <is>
-          <t>Phase 4</t>
+          <t>Phase 1</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>MEP &amp; Finishes</t>
+          <t>Shop Drawings &amp; Fabrication</t>
         </is>
       </c>
       <c r="E45" s="17" t="inlineStr">
         <is>
-          <t>4 months</t>
+          <t>2 months</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>25% overlap with structure</t>
+          <t>Before on-site work</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="17" t="inlineStr">
         <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Foundation &amp; Columns</t>
+        </is>
+      </c>
+      <c r="E46" s="17" t="inlineStr">
+        <is>
+          <t>3 months</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Concurrent with fabrication</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="17" t="inlineStr">
+        <is>
+          <t>Phase 3</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Deck Installation (7 floors)</t>
+        </is>
+      </c>
+      <c r="E47" s="17" t="inlineStr">
+        <is>
+          <t>9 months</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>1.3 months per floor</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="17" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>MEP &amp; Finishes</t>
+        </is>
+      </c>
+      <c r="E48" s="17" t="inlineStr">
+        <is>
+          <t>4 months</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>25% overlap with structure</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="17" t="inlineStr">
+        <is>
           <t>Total Duration</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>Ground to CO</t>
         </is>
       </c>
-      <c r="E46" s="17" t="inlineStr">
+      <c r="E49" s="17" t="inlineStr">
         <is>
           <t>18 months</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F49" t="inlineStr">
         <is>
           <t>6 months faster than traditional</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="18" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="18" t="inlineStr">
         <is>
           <t>SUBMITTAL REQUIREMENTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>1. Complete project pricing breakdown</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>2. Shop drawings and engineering calculations</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>3. Product data sheets and specifications</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>4. Quality control procedures</t>
+          <t>1. Complete project pricing breakdown</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>5. Installation schedule and sequence</t>
+          <t>2. Shop drawings and engineering calculations</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>6. Crane and equipment requirements</t>
+          <t>3. Product data sheets and specifications</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>7. Testing and inspection protocols</t>
+          <t>4. Quality control procedures</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>8. Warranty information (minimum 2 years)</t>
+          <t>5. Installation schedule and sequence</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>9. References from similar high-rise projects</t>
+          <t>6. Crane and equipment requirements</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
+          <t>7. Testing and inspection protocols</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>8. Warranty information (minimum 2 years)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>9. References from similar high-rise projects</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
           <t>10. Insurance certificates</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="43">
+  <mergeCells count="45">
     <mergeCell ref="B11:D11"/>
-    <mergeCell ref="B42:D42"/>
-    <mergeCell ref="A48:H48"/>
-    <mergeCell ref="F42:H42"/>
     <mergeCell ref="A15:H15"/>
     <mergeCell ref="A59:H59"/>
     <mergeCell ref="F45:H45"/>
     <mergeCell ref="A24:H24"/>
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="A51:H51"/>
+    <mergeCell ref="A60:H60"/>
     <mergeCell ref="B13:D13"/>
-    <mergeCell ref="B44:D44"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A61:H61"/>
     <mergeCell ref="A6:H6"/>
+    <mergeCell ref="F47:H47"/>
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="F46:H46"/>
+    <mergeCell ref="A25:H25"/>
     <mergeCell ref="A54:H54"/>
+    <mergeCell ref="B49:D49"/>
     <mergeCell ref="B9:D9"/>
-    <mergeCell ref="F43:H43"/>
+    <mergeCell ref="F48:H48"/>
     <mergeCell ref="A18:H18"/>
-    <mergeCell ref="A50:H50"/>
     <mergeCell ref="A56:H56"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A21:H21"/>
     <mergeCell ref="A26:H26"/>
     <mergeCell ref="A55:H55"/>
     <mergeCell ref="B45:D45"/>
+    <mergeCell ref="F49:H49"/>
     <mergeCell ref="A57:H57"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="F44:H44"/>
     <mergeCell ref="A23:H23"/>
+    <mergeCell ref="B47:D47"/>
     <mergeCell ref="A22:H22"/>
     <mergeCell ref="A17:H17"/>
     <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A62:H62"/>
     <mergeCell ref="A53:H53"/>
     <mergeCell ref="B46:D46"/>
     <mergeCell ref="A20:H20"/>
-    <mergeCell ref="A52:H52"/>
+    <mergeCell ref="A43:H43"/>
+    <mergeCell ref="A28:H28"/>
     <mergeCell ref="A19:H19"/>
-    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="A58:H58"/>
     <mergeCell ref="B12:D12"/>
-    <mergeCell ref="A58:H58"/>
-    <mergeCell ref="A40:H40"/>
+    <mergeCell ref="B48:D48"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -38513,7 +38561,7 @@
         </is>
       </c>
       <c r="C20" s="19" t="n">
-        <v>8.77</v>
+        <v>7.89</v>
       </c>
       <c r="D20" s="12" t="n">
         <v>108675</v>
@@ -38522,9 +38570,9 @@
         <f>C20*D20</f>
         <v/>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Same</t>
+      <c r="F20" s="89" t="inlineStr">
+        <is>
+          <t>10% savings - embedded in slab</t>
         </is>
       </c>
     </row>
@@ -38567,7 +38615,7 @@
         </is>
       </c>
       <c r="C22" s="19" t="n">
-        <v>13.15</v>
+        <v>11.84</v>
       </c>
       <c r="D22" s="12" t="n">
         <v>108675</v>
@@ -38576,9 +38624,9 @@
         <f>C22*D22</f>
         <v/>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Same</t>
+      <c r="F22" s="89" t="inlineStr">
+        <is>
+          <t>10% savings - conduits in slab</t>
         </is>
       </c>
     </row>
@@ -38766,7 +38814,7 @@
       </c>
       <c r="F32" s="93" t="inlineStr">
         <is>
-          <t>4.3% reduction</t>
+          <t>5.4% reduction</t>
         </is>
       </c>
     </row>

</xml_diff>